<commit_message>
feat: add cloud-ready recruiting operations and campus sources
</commit_message>
<xml_diff>
--- a/项目管理/项目推进台账.xlsx
+++ b/项目管理/项目推进台账.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rbe20885f926c44c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="Rc46a40305a3f48ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="R589df6654730421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R78ce26749b294ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="Rc400f40606a0498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="R9b2caf8a1f684ad0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -636,7 +636,7 @@
         <x:v>面向上海立信会计金融学院学生的非官方就业信息服务｜最后更新：2026-08-26</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>面向上海立信会计金融学院学生的非官方就业信息服务｜最后更新：2026-09-04</x:v>
+        <x:v>2026-09-05</x:v>
       </x:c>
       <x:c r="C2" s="7"/>
       <x:c r="D2" s="7"/>
@@ -679,7 +679,7 @@
         <x:v>可信采集 → 人工核验 → 内容分发</x:v>
       </x:c>
       <x:c r="C5" s="16" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>0</x:v>
@@ -2184,40 +2184,100 @@
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="36"/>
-      <x:c r="B43" s="37"/>
-      <x:c r="C43" s="37"/>
-      <x:c r="D43" s="37"/>
-      <x:c r="E43" s="37"/>
-      <x:c r="F43" s="37"/>
-      <x:c r="G43" s="37"/>
-      <x:c r="H43" s="37"/>
-      <x:c r="I43" s="37"/>
-      <x:c r="J43" s="38"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="36"/>
-      <x:c r="B44" s="37"/>
-      <x:c r="C44" s="37"/>
-      <x:c r="D44" s="37"/>
-      <x:c r="E44" s="37"/>
-      <x:c r="F44" s="37"/>
-      <x:c r="G44" s="37"/>
-      <x:c r="H44" s="37"/>
-      <x:c r="I44" s="37"/>
-      <x:c r="J44" s="38"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="36"/>
-      <x:c r="B45" s="37"/>
-      <x:c r="C45" s="37"/>
-      <x:c r="D45" s="37"/>
-      <x:c r="E45" s="37"/>
-      <x:c r="F45" s="37"/>
-      <x:c r="G45" s="37"/>
-      <x:c r="H45" s="37"/>
-      <x:c r="I45" s="37"/>
-      <x:c r="J45" s="38"/>
+      <x:c r="A43" s="36" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B43" s="37" t="str">
+        <x:v>2026-09-05</x:v>
+      </x:c>
+      <x:c r="C43" s="37" t="str">
+        <x:v>可信交付 / 发布安全</x:v>
+      </x:c>
+      <x:c r="D43" s="37" t="str">
+        <x:v>证据、版本与发布门槛 v1.1</x:v>
+      </x:c>
+      <x:c r="E43" s="37" t="str">
+        <x:v>正文提取优先文章区域，区分公告发布时间与拉取时间；AI 字段规范化并分开公告标题和岗位名称；人工核验、岗位事实与草稿按版本绑定。</x:v>
+      </x:c>
+      <x:c r="F43" s="37" t="str">
+        <x:v>采集器 / AI 结构化 / 审核 / 内容队列 / 启动脚本</x:v>
+      </x:c>
+      <x:c r="G43" s="37" t="str">
+        <x:v>新增正文清洗、时效、版本失效、批量任务和表单错误回归测试；本轮 178 项测试分组通过，PowerShell 脚本语法通过。</x:v>
+      </x:c>
+      <x:c r="H43" s="37" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I43" s="37" t="str">
+        <x:v>图片和扫描 PDF 尚未自动解析；真实来源、公众号粘贴及同事干净电脑启动仍需运营实测。</x:v>
+      </x:c>
+      <x:c r="J43" s="38" t="str">
+        <x:v>使用 10 类公告样本及一周小范围试运行，记录准确率、人工耗时与启动结果。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="48" customHeight="1">
+      <x:c r="A44" s="49" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B44" s="34" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="C44" s="34" t="str">
+        <x:v>来源扩充</x:v>
+      </x:c>
+      <x:c r="D44" s="34" t="str">
+        <x:v>高校就业网公开试采适配</x:v>
+      </x:c>
+      <x:c r="E44" s="34" t="str">
+        <x:v>新增 8 个 B 类候选来源；完成交大与上财公开 JSON 适配、稳定职位身份与全详情失败识别。</x:v>
+      </x:c>
+      <x:c r="F44" s="34" t="str">
+        <x:v>来源目录 / 采集器 / 去重与来源健康</x:v>
+      </x:c>
+      <x:c r="G44" s="34" t="str">
+        <x:v>离线适配测试 17 项通过；全量 pytest 272 项通过。</x:v>
+      </x:c>
+      <x:c r="H44" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I44" s="34" t="str">
+        <x:v>交大、上财保持 B 类禁用；华东理工为校内访问限制；未自动发布或自动启用。</x:v>
+      </x:c>
+      <x:c r="J44" s="35" t="str">
+        <x:v>完成连续 3 次隔离试采和人工确认后，再决定是否升 A 类。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="48" customHeight="1">
+      <x:c r="A45" s="49" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B45" s="34" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="C45" s="34" t="str">
+        <x:v>来源试采</x:v>
+      </x:c>
+      <x:c r="D45" s="34" t="str">
+        <x:v>B 类候选输入隔离提取</x:v>
+      </x:c>
+      <x:c r="E45" s="34" t="str">
+        <x:v>新增 B 类高校来源的隔离候选提取器；仅保留明确上海且具有官方投递链接或邮箱证据的职位，不写正式岗位库。</x:v>
+      </x:c>
+      <x:c r="F45" s="34" t="str">
+        <x:v>B 类试采 / 地点筛选 / 投递证据</x:v>
+      </x:c>
+      <x:c r="G45" s="34" t="str">
+        <x:v>定向测试通过；全量 pytest 273 项通过；交大首轮筛出 1 条合格候选，上财首轮为 0 条。</x:v>
+      </x:c>
+      <x:c r="H45" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I45" s="34" t="str">
+        <x:v>试采不改变 B 类禁用状态；一次结果不代表可自动采集，仍需连续 3 次和人工确认。</x:v>
+      </x:c>
+      <x:c r="J45" s="35" t="str">
+        <x:v>记录后续两次隔离试采，并人工核验交大候选的原文与投递入口。</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="36"/>

</xml_diff>

<commit_message>
feat: expand B-grade intake and add four public source adapters
Add bounded NCSS and university/association trials, manual B intake evidence gates, collection safeguards, and longer AI text read timeouts. Include regression coverage, implementation reports, and project ledger; exclude all local backups and runtime data.
</commit_message>
<xml_diff>
--- a/项目管理/项目推进台账.xlsx
+++ b/项目管理/项目推进台账.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R78ce26749b294ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="Rc400f40606a0498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="R9b2caf8a1f684ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rf8194f3ae066486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="Ra4feb8068d9148c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="R0d4d3f1d43c54477"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -221,7 +224,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="83">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -392,6 +395,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2279,29 +2285,69 @@
         <x:v>记录后续两次隔离试采，并人工核验交大候选的原文与投递入口。</x:v>
       </x:c>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="36"/>
-      <x:c r="B46" s="37"/>
-      <x:c r="C46" s="37"/>
-      <x:c r="D46" s="37"/>
-      <x:c r="E46" s="37"/>
-      <x:c r="F46" s="37"/>
-      <x:c r="G46" s="37"/>
-      <x:c r="H46" s="37"/>
-      <x:c r="I46" s="37"/>
-      <x:c r="J46" s="38"/>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="36"/>
-      <x:c r="B47" s="37"/>
-      <x:c r="C47" s="37"/>
-      <x:c r="D47" s="37"/>
-      <x:c r="E47" s="37"/>
-      <x:c r="F47" s="37"/>
-      <x:c r="G47" s="37"/>
-      <x:c r="H47" s="37"/>
-      <x:c r="I47" s="37"/>
-      <x:c r="J47" s="38"/>
+    <x:row r="46" ht="100" customHeight="1">
+      <x:c r="A46" s="49" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B46" s="83" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C46" s="34" t="str">
+        <x:v>岗位准入 / 人工筛选</x:v>
+      </x:c>
+      <x:c r="D46" s="34" t="str">
+        <x:v>B级岗位人工筛选池</x:v>
+      </x:c>
+      <x:c r="E46" s="34" t="str">
+        <x:v>重新划分岗位初筛：符合上海、在招、投递与完整原文条件但学生受众不明的线索进入B级待核验。官网复核后6条存量C迁B，实际A38/B6/C69/D64。</x:v>
+      </x:c>
+      <x:c r="F46" s="34" t="str">
+        <x:v>初筛 / 试点入库 / 人审 / 内容队列 / 历史迁移</x:v>
+      </x:c>
+      <x:c r="G46" s="34" t="str">
+        <x:v>全量pytest 710项通过；6条B在页面展示；官网复核、两次备份、审核审计、数据库完整性检查通过。</x:v>
+      </x:c>
+      <x:c r="H46" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I46" s="34" t="str">
+        <x:v>B级仍需人工确认受众，未确认不能发布；来源级别与岗位等级分开；多岗位证据隔离，保留既有人工处理记录。</x:v>
+      </x:c>
+      <x:c r="J46" s="35" t="str">
+        <x:v>逐条筛选6条B岗位，补齐受众与事实后终审；继续观察日均新增和合格率。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="150" customHeight="1">
+      <x:c r="A47" s="49" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B47" s="83" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C47" s="34" t="str">
+        <x:v>来源试采 / 待核验入库</x:v>
+      </x:c>
+      <x:c r="D47" s="34" t="str">
+        <x:v>四个B类公开来源真实试跑</x:v>
+      </x:c>
+      <x:c r="E47" s="34" t="str">
+        <x:v>NCSS上海、上海工程技术大学、上海应用技术大学、上海注协各试采30条列表、10条详情。成功详情9/9/10/10，新增待核验记录9/6/1/0，共16条（11A、5B）。真实岗位总计193条：A49/B11/C69/D64。</x:v>
+      </x:c>
+      <x:c r="F47" s="34" t="str">
+        <x:v>四源适配 / B类隔离试采 / 待核验入库 / 来源监控</x:v>
+      </x:c>
+      <x:c r="G47" s="34" t="str">
+        <x:v>全量pytest 785项通过（1条既有警告）；重复导入新增0、更新0，保持9/6/1条；SQLite完整性检查通过；试点与岗位页HTTP200。</x:v>
+      </x:c>
+      <x:c r="H47" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I47" s="34" t="str">
+        <x:v>四个来源仍为B类且自动采集禁用，未自动发布。16为记录数，按公司与标题粗合并约13组，待人工去重；单轮结果不能视为稳定日均产出。上海注协缺明确工作地点，部分另受经验或过期限制。</x:v>
+      </x:c>
+      <x:c r="J47" s="35" t="str">
+        <x:v>人工核验16条新增记录的上海地点、学生受众、在招状态与投递入口，核对跨来源同名记录；继续连续隔离试采后，再决定来源准入。</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="36"/>

</xml_diff>

<commit_message>
feat: add screenshot-to-content workflow with AI prefill and guided review
</commit_message>
<xml_diff>
--- a/项目管理/项目推进台账.xlsx
+++ b/项目管理/项目推进台账.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rf8194f3ae066486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="Ra4feb8068d9148c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="R0d4d3f1d43c54477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R06d9312354bc4b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="R9ef73b38b6364b96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="Rfbf9edde138b4d76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2349,41 +2349,101 @@
         <x:v>人工核验16条新增记录的上海地点、学生受众、在招状态与投递入口，核对跨来源同名记录；继续连续隔离试采后，再决定来源准入。</x:v>
       </x:c>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="36"/>
-      <x:c r="B48" s="37"/>
-      <x:c r="C48" s="37"/>
-      <x:c r="D48" s="37"/>
-      <x:c r="E48" s="37"/>
-      <x:c r="F48" s="37"/>
-      <x:c r="G48" s="37"/>
-      <x:c r="H48" s="37"/>
-      <x:c r="I48" s="37"/>
-      <x:c r="J48" s="38"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="36"/>
-      <x:c r="B49" s="37"/>
-      <x:c r="C49" s="37"/>
-      <x:c r="D49" s="37"/>
-      <x:c r="E49" s="37"/>
-      <x:c r="F49" s="37"/>
-      <x:c r="G49" s="37"/>
-      <x:c r="H49" s="37"/>
-      <x:c r="I49" s="37"/>
-      <x:c r="J49" s="38"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="36"/>
-      <x:c r="B50" s="37"/>
-      <x:c r="C50" s="37"/>
-      <x:c r="D50" s="37"/>
-      <x:c r="E50" s="37"/>
-      <x:c r="F50" s="37"/>
-      <x:c r="G50" s="37"/>
-      <x:c r="H50" s="37"/>
-      <x:c r="I50" s="37"/>
-      <x:c r="J50" s="38"/>
+    <x:row r="48" ht="150" customHeight="1">
+      <x:c r="A48" s="49" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B48" s="83" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C48" s="34" t="str">
+        <x:v>截图工作区 / 双渠道内容</x:v>
+      </x:c>
+      <x:c r="D48" s="34" t="str">
+        <x:v>截图转微信群与公众号内容</x:v>
+      </x:c>
+      <x:c r="E48" s="34" t="str">
+        <x:v>新增截图上传、长图分片、可恢复识别、原图校对、独立岗位与公共条件编辑。人工核验和审核后，按同一事实快照生成微信群与公众号稿；事实修改立即使旧稿失效。</x:v>
+      </x:c>
+      <x:c r="F48" s="34" t="str">
+        <x:v>截图上传 / OCR与任务 / 字段校对 / 审核 / 双渠道复制</x:v>
+      </x:c>
+      <x:c r="G48" s="34" t="str">
+        <x:v>全量pytest 1035项通过（1条既有弃用警告，59.53秒）。隔离浏览器上传、校对、87分审核及两渠道复制载荷通过；390px无横向溢出、控制台0错误。真实API 6组合成材料中4组质量通过。205条真实业务记录逐列未变。</x:v>
+      </x:c>
+      <x:c r="H48" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I48" s="34" t="str">
+        <x:v>本地已完成，真实材料待试用。复杂多岗证据拒绝、模糊邮箱及重试超时需人工；不是6/6通过，不代表OCR准确率。真实微信截图、微信后台富文本粘贴和PostgreSQL未实测；未云部署，不自动发微信。</x:v>
+      </x:c>
+      <x:c r="J48" s="35" t="str">
+        <x:v>使用客户真实截图试用，补多岗证据与模糊材料人工校对。实测微信公众号编辑器和PostgreSQL后，再决定云部署。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="150" customHeight="1">
+      <x:c r="A49" s="49" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B49" s="83" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C49" s="34" t="str">
+        <x:v>截图识别 / AI预填</x:v>
+      </x:c>
+      <x:c r="D49" s="34" t="str">
+        <x:v>结构化预填与局部恢复</x:v>
+      </x:c>
+      <x:c r="E49" s="34" t="str">
+        <x:v>截图字段按固定结构自动预填。首次不合格最多修复一次，保留有效字段并定位疑点。增加原文未提供确认、各岗条件校对及重新提取后旧审核失效。</x:v>
+      </x:c>
+      <x:c r="F49" s="34" t="str">
+        <x:v>AI配置 / 提取任务 / 原文证据 / 字段校对 / 审核与复制</x:v>
+      </x:c>
+      <x:c r="G49" s="34" t="str">
+        <x:v>全量1176项通过（1条既有警告，118.42秒）。真实图预填0至15项，2次文本调用、复用2片OCR。205条真实岗位及来源、审核、分发逐行未变。</x:v>
+      </x:c>
+      <x:c r="H49" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I49" s="34" t="str">
+        <x:v>真实图仍有4处疑点（1处不明确、3处冲突），未审核、未建岗位、未发布。全程约142秒含排队，不代表提速。材料主要面向硕博，需核对学生适配。</x:v>
+      </x:c>
+      <x:c r="J49" s="35" t="str">
+        <x:v>逐项处理真实截图疑点，补齐来源及官方入口后人工复核。继续观察不同海报的字段命中、耗时和岗位条件边界。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="150" customHeight="1">
+      <x:c r="A50" s="49" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B50" s="83" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C50" s="34" t="str">
+        <x:v>截图转内容 / 问题优先审核</x:v>
+      </x:c>
+      <x:c r="D50" s="34" t="str">
+        <x:v>摘要校对与一次人工终审</x:v>
+      </x:c>
+      <x:c r="E50" s="34" t="str">
+        <x:v>摘要及双渠道预览优先，完整字段默认收起。必填、选填与条件必填分开；红标说明原因并定位。一次明确确认替代逐项勾选和手填质量分，失败保留草稿。</x:v>
+      </x:c>
+      <x:c r="F50" s="34" t="str">
+        <x:v>AI字段整理 / 原文证据 / 截图校对 / 审核 / 双渠道复制</x:v>
+      </x:c>
+      <x:c r="G50" s="34" t="str">
+        <x:v>全量1383项通过（1条既有警告，126.57秒）。浏览器一键生成、三错误保留输入、390px无横向溢出及旧稿失效通过。205条真实岗位及来源、审核、分发、原图记录逐列未变。</x:v>
+      </x:c>
+      <x:c r="H50" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I50" s="34" t="str">
+        <x:v>只对当前截图终审证明替代数值门槛，不提高质量分；其他岗位仍保留70分规则。未重跑真实AI、未代审真实材料，未实测微信后台粘贴和云端PostgreSQL；不自动发送。</x:v>
+      </x:c>
+      <x:c r="J50" s="35" t="str">
+        <x:v>使用新页面处理真实材料；按需点击AI补全与整理。补齐实际缺失的来源、岗位和投递依据，再人工核验；观察多岗位、长图的耗时与问题提示。</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="36"/>

</xml_diff>

<commit_message>
fix: accept explicitly unspecified screenshot deadlines
Treat whole-clause no-deadline statements as valid absence, clarify optional deadline input, add 16 regression cases, and record the verified fix in the project ledger.
</commit_message>
<xml_diff>
--- a/项目管理/项目推进台账.xlsx
+++ b/项目管理/项目推进台账.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R06d9312354bc4b16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="R9ef73b38b6364b96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="Rfbf9edde138b4d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R508c2c2890054039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新台账" sheetId="2" r:id="R7cde0c62a9c44e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="登记规范" sheetId="3" r:id="Ra033a3c8ce19412b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2445,17 +2445,37 @@
         <x:v>使用新页面处理真实材料；按需点击AI补全与整理。补齐实际缺失的来源、岗位和投递依据，再人工核验；观察多岗位、长图的耗时与问题提示。</x:v>
       </x:c>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="36"/>
-      <x:c r="B51" s="37"/>
-      <x:c r="C51" s="37"/>
-      <x:c r="D51" s="37"/>
-      <x:c r="E51" s="37"/>
-      <x:c r="F51" s="37"/>
-      <x:c r="G51" s="37"/>
-      <x:c r="H51" s="37"/>
-      <x:c r="I51" s="37"/>
-      <x:c r="J51" s="38"/>
+    <x:row r="51" ht="150" customHeight="1">
+      <x:c r="A51" s="49" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B51" s="83" t="d">
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C51" s="34" t="str">
+        <x:v>截图校对 / 截止日期</x:v>
+      </x:c>
+      <x:c r="D51" s="34" t="str">
+        <x:v>未公布截止日期误拦截修复</x:v>
+      </x:c>
+      <x:c r="E51" s="34" t="str">
+        <x:v>原文“公告未明确统一截止时间”被误判为日期损坏，空日期仍被拦截。现按完整语句识别未公布说明，截止日期标为选填并提示可留空。</x:v>
+      </x:c>
+      <x:c r="F51" s="34" t="str">
+        <x:v>截图审核规则 / 原文证据 / 人工校对页面</x:v>
+      </x:c>
+      <x:c r="G51" s="34" t="str">
+        <x:v>新增16项回归，相关156项及全量1399项通过（1条既有警告）。独立246组边界断言通过。本地HTTP200已加载选填提示。</x:v>
+      </x:c>
+      <x:c r="H51" s="34" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="I51" s="34" t="str">
+        <x:v>只识别完整无期限语句，不跳过原文日期限制。未调用真实AI、未代审或发布；另一台电脑需同步版本。</x:v>
+      </x:c>
+      <x:c r="J51" s="35" t="str">
+        <x:v>按选填提示保留空日期，补齐其余问题后人工复核。继续观察日期缺失、缺年、无效、过期及冲突提示。</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="36"/>

</xml_diff>